<commit_message>
add parameter idenfication and sim code for 18650PF battery
</commit_message>
<xml_diff>
--- a/data/HP02R0301A2 data_SOC vs Vth_18650-30Q_extracted_Fig_03_park2025RefinedAircooled_xin_20251208.xlsx
+++ b/data/HP02R0301A2 data_SOC vs Vth_18650-30Q_extracted_Fig_03_park2025RefinedAircooled_xin_20251208.xlsx
@@ -5,16 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\eBATS\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\HAUST\02 HP02_HNPRJ_2024 eVTOL BTMS\01_proposal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8636F959-846F-4F5F-9D7B-DA55880BF20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{848A2BDB-0B1D-4D21-A0C2-B859AEE04130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="345" yWindow="1680" windowWidth="16410" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5C" sheetId="1" r:id="rId1"/>
-    <sheet name="3.3C_x0009_" sheetId="2" r:id="rId2"/>
+    <sheet name="3.3C" sheetId="2" r:id="rId2"/>
     <sheet name="1.7C" sheetId="3" r:id="rId3"/>
     <sheet name="1C" sheetId="4" r:id="rId4"/>
   </sheets>
@@ -33,7 +33,7 @@
     <t>SOC</t>
   </si>
   <si>
-    <t>Vth</t>
+    <t>V_out</t>
   </si>
 </sst>
 </file>
@@ -85,7 +85,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -93,9 +93,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1373,7 +1370,7 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1865,7 +1862,7 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>